<commit_message>
inserção do mes de junho no banco de dados
</commit_message>
<xml_diff>
--- a/data/input/metas.xlsx
+++ b/data/input/metas.xlsx
@@ -164,7 +164,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.45703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -176,251 +176,187 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>2874.88</v>
-      </c>
+        <v>46174</v>
+      </c>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
-        <v>46144</v>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>4633.35</v>
-      </c>
+        <v>46175</v>
+      </c>
+      <c r="B3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
-        <v>46145</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>4467.71</v>
-      </c>
+        <v>46176</v>
+      </c>
+      <c r="B4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
-        <v>46146</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>2465.12</v>
-      </c>
+        <v>46177</v>
+      </c>
+      <c r="B5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
-        <v>46147</v>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>2649.56</v>
-      </c>
+        <v>46178</v>
+      </c>
+      <c r="B6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
-        <v>46148</v>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>2953.77</v>
-      </c>
+        <v>46179</v>
+      </c>
+      <c r="B7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
-        <v>46149</v>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>2785.57</v>
-      </c>
+        <v>46180</v>
+      </c>
+      <c r="B8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>2874.88</v>
-      </c>
+        <v>46181</v>
+      </c>
+      <c r="B9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
-        <v>46151</v>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>4633.35</v>
-      </c>
+        <v>46182</v>
+      </c>
+      <c r="B10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>4467.71</v>
-      </c>
+        <v>46183</v>
+      </c>
+      <c r="B11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
-        <v>46153</v>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>2465.12</v>
-      </c>
+        <v>46184</v>
+      </c>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
-        <v>46154</v>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>2649.56</v>
-      </c>
+        <v>46185</v>
+      </c>
+      <c r="B13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="n">
-        <v>46155</v>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>2953.77</v>
-      </c>
+        <v>46186</v>
+      </c>
+      <c r="B14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>2785.57</v>
-      </c>
+        <v>46187</v>
+      </c>
+      <c r="B15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="n">
-        <v>46157</v>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>2874.88</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="B16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="n">
-        <v>46158</v>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>4633.35</v>
-      </c>
+        <v>46189</v>
+      </c>
+      <c r="B17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="n">
-        <v>46159</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>4467.71</v>
-      </c>
+        <v>46190</v>
+      </c>
+      <c r="B18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="n">
-        <v>46160</v>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>2465.12</v>
-      </c>
+        <v>46191</v>
+      </c>
+      <c r="B19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>2649.56</v>
-      </c>
+        <v>46192</v>
+      </c>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="n">
-        <v>46162</v>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>2953.77</v>
-      </c>
+        <v>46193</v>
+      </c>
+      <c r="B21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
-        <v>46163</v>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>2785.57</v>
-      </c>
+        <v>46194</v>
+      </c>
+      <c r="B22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>2874.88</v>
-      </c>
+        <v>46195</v>
+      </c>
+      <c r="B23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
-        <v>46165</v>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>4633.35</v>
-      </c>
+        <v>46196</v>
+      </c>
+      <c r="B24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
-        <v>46166</v>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>4467.71</v>
-      </c>
+        <v>46197</v>
+      </c>
+      <c r="B25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
-        <v>46167</v>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>2465.12</v>
-      </c>
+        <v>46198</v>
+      </c>
+      <c r="B26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
-        <v>46168</v>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>2649.56</v>
-      </c>
+        <v>46199</v>
+      </c>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
-        <v>46169</v>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>2953.77</v>
-      </c>
+        <v>46200</v>
+      </c>
+      <c r="B28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
-        <v>46170</v>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>2785.57</v>
-      </c>
+        <v>46201</v>
+      </c>
+      <c r="B29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>2874.88</v>
-      </c>
+        <v>46202</v>
+      </c>
+      <c r="B30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>4633.35</v>
-      </c>
+        <v>46203</v>
+      </c>
+      <c r="B31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B32" s="4" t="n">
-        <v>4467.71</v>
-      </c>
+      <c r="A32" s="3"/>
+      <c r="B32" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
alteração nos scripts de inserir mes e inserir meta
</commit_message>
<xml_diff>
--- a/data/input/metas.xlsx
+++ b/data/input/metas.xlsx
@@ -164,7 +164,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultColWidth="14.45703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.46484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -178,181 +178,241 @@
       <c r="A2" s="3" t="n">
         <v>46174</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="B2" s="4" t="n">
+        <v>2441.73</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
         <v>46175</v>
       </c>
-      <c r="B3" s="4"/>
+      <c r="B3" s="4" t="n">
+        <v>2595.82</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
         <v>46176</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="4" t="n">
+        <v>3050.37</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
         <v>46177</v>
       </c>
-      <c r="B5" s="4"/>
+      <c r="B5" s="4" t="n">
+        <v>2625.01</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
         <v>46178</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="4" t="n">
+        <v>2871.52</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
         <v>46179</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="4" t="n">
+        <v>4812.18</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
         <v>46180</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="4" t="n">
+        <v>4517.61</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
         <v>46181</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="4" t="n">
+        <v>2441.73</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
         <v>46182</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="4" t="n">
+        <v>2595.82</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
         <v>46183</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="4" t="n">
+        <v>3050.37</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
         <v>46184</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="4" t="n">
+        <v>2625.01</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
         <v>46185</v>
       </c>
-      <c r="B13" s="4"/>
+      <c r="B13" s="4" t="n">
+        <v>2871.52</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="n">
         <v>46186</v>
       </c>
-      <c r="B14" s="4"/>
+      <c r="B14" s="4" t="n">
+        <v>4812.18</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="n">
         <v>46187</v>
       </c>
-      <c r="B15" s="4"/>
+      <c r="B15" s="4" t="n">
+        <v>4517.61</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="n">
         <v>46188</v>
       </c>
-      <c r="B16" s="4"/>
+      <c r="B16" s="4" t="n">
+        <v>2441.73</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="n">
         <v>46189</v>
       </c>
-      <c r="B17" s="4"/>
+      <c r="B17" s="4" t="n">
+        <v>2595.82</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="n">
         <v>46190</v>
       </c>
-      <c r="B18" s="4"/>
+      <c r="B18" s="4" t="n">
+        <v>3050.37</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="n">
         <v>46191</v>
       </c>
-      <c r="B19" s="4"/>
+      <c r="B19" s="4" t="n">
+        <v>2625.01</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="n">
         <v>46192</v>
       </c>
-      <c r="B20" s="4"/>
+      <c r="B20" s="4" t="n">
+        <v>2871.52</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="n">
         <v>46193</v>
       </c>
-      <c r="B21" s="4"/>
+      <c r="B21" s="4" t="n">
+        <v>4812.18</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
         <v>46194</v>
       </c>
-      <c r="B22" s="4"/>
+      <c r="B22" s="4" t="n">
+        <v>4517.61</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
         <v>46195</v>
       </c>
-      <c r="B23" s="4"/>
+      <c r="B23" s="4" t="n">
+        <v>2441.73</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
         <v>46196</v>
       </c>
-      <c r="B24" s="4"/>
+      <c r="B24" s="4" t="n">
+        <v>2595.82</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
         <v>46197</v>
       </c>
-      <c r="B25" s="4"/>
+      <c r="B25" s="4" t="n">
+        <v>3050.37</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
         <v>46198</v>
       </c>
-      <c r="B26" s="4"/>
+      <c r="B26" s="4" t="n">
+        <v>2625.01</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
         <v>46199</v>
       </c>
-      <c r="B27" s="4"/>
+      <c r="B27" s="4" t="n">
+        <v>2871.52</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
         <v>46200</v>
       </c>
-      <c r="B28" s="4"/>
+      <c r="B28" s="4" t="n">
+        <v>4812.18</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
         <v>46201</v>
       </c>
-      <c r="B29" s="4"/>
+      <c r="B29" s="4" t="n">
+        <v>4517.61</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="n">
         <v>46202</v>
       </c>
-      <c r="B30" s="4"/>
+      <c r="B30" s="4" t="n">
+        <v>2441.73</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
         <v>46203</v>
       </c>
-      <c r="B31" s="4"/>
+      <c r="B31" s="4" t="n">
+        <v>2595.82</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>

</xml_diff>